<commit_message>
Modified layout and axis format of scatter charts.
Content remains the same.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/WLIsoCheckTemplate.xlsx
+++ b/src/main/resources/static/WLIsoCheckTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pf\IntelliJ\ws\aqa\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F64FBDB1-81BA-4395-88C6-794E8F3F7BA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E2D3CA-9F85-4B34-BEE7-4272916FF625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4125" yWindow="495" windowWidth="46740" windowHeight="13185" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-345" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SNCImport" sheetId="6" r:id="rId1"/>
@@ -1362,12 +1362,9 @@
     <a:solidFill>
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="tx1"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -1736,12 +1733,9 @@
     <a:solidFill>
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
+        <a:schemeClr val="tx1"/>
       </a:solidFill>
       <a:round/>
     </a:ln>
@@ -2882,15 +2876,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>190499</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>409575</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>19049</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2919,16 +2913,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>419100</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>180974</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>9524</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>1680</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>152399</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>883023</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>

<commit_message>
Finished making IsoTable processing optional.
Also, several minor spreadsheet tweaks.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/WLIsoCheckTemplate.xlsx
+++ b/src/main/resources/static/WLIsoCheckTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pf\IntelliJ\ws\aqa\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E2D3CA-9F85-4B34-BEE7-4272916FF625}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083A60B7-DFC4-434F-AD66-5CCBC434746D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-345" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SNCImport" sheetId="6" r:id="rId1"/>
@@ -518,9 +518,6 @@
     <t>Table - Gantry Iso Z (mm)</t>
   </si>
   <si>
-    <t>Gantry Flex (mm)</t>
-  </si>
-  <si>
     <t>Col-Gantry misalignment (mm)</t>
   </si>
   <si>
@@ -613,7 +610,10 @@
     <t>Winston-Lutz Field Data</t>
   </si>
   <si>
-    <t>To re-calculate spreadsheet in Excel, use CTRL-ALT-SHIFT-F9 and then run the solver on each of the Analysis and Collimator sheets.</t>
+    <t>To re-calculate spreadsheet in Excel, use CTRL-ALT-F9 and then run the solver on each of the Analysis and Collimator sheets.</t>
+  </si>
+  <si>
+    <t>Gantry Flex (mm)</t>
   </si>
 </sst>
 </file>
@@ -3304,7 +3304,7 @@
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="33" t="s">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="C7" s="34" t="str">
         <f>Analysis!O3</f>
@@ -3313,7 +3313,7 @@
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="33" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C8" s="34" t="e">
         <f>Analysis!P3</f>
@@ -3322,7 +3322,7 @@
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="33" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C9" s="34" t="str">
         <f>Analysis!T1</f>
@@ -3331,7 +3331,7 @@
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="33" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C10" s="34">
         <f>SQRT(Analysis!R12)</f>
@@ -3340,7 +3340,7 @@
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B11" s="33" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C11" s="34">
         <f>Analysis!O8</f>
@@ -3349,7 +3349,7 @@
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="33" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C12" s="34">
         <f>Collimator!L2</f>
@@ -3392,13 +3392,13 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1" s="38" t="s">
+        <v>127</v>
+      </c>
+      <c r="C1" s="38" t="s">
         <v>128</v>
-      </c>
-      <c r="C1" s="38" t="s">
-        <v>129</v>
       </c>
       <c r="D1" s="38"/>
       <c r="E1" s="38"/>
@@ -3491,7 +3491,7 @@
         <v>21</v>
       </c>
       <c r="W2" s="38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="X2" s="38" t="s">
         <v>97</v>
@@ -3502,13 +3502,13 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D3" s="38">
         <v>-1</v>
@@ -3565,27 +3565,27 @@
         <v>-1</v>
       </c>
       <c r="V3" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W3" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X3" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y3" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D4" s="38">
         <v>-1</v>
@@ -3642,27 +3642,27 @@
         <v>-1</v>
       </c>
       <c r="V4" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W4" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X4" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y4" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D5" s="38">
         <v>-1</v>
@@ -3719,27 +3719,27 @@
         <v>-1</v>
       </c>
       <c r="V5" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W5" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X5" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y5" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D6" s="38">
         <v>-1</v>
@@ -3796,27 +3796,27 @@
         <v>-1</v>
       </c>
       <c r="V6" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W6" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X6" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y6" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7" s="38">
         <v>-1</v>
@@ -3873,27 +3873,27 @@
         <v>-1</v>
       </c>
       <c r="V7" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W7" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X7" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y7" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D8" s="38">
         <v>-1</v>
@@ -3950,27 +3950,27 @@
         <v>-1</v>
       </c>
       <c r="V8" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W8" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X8" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y8" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D9" s="38">
         <v>-1</v>
@@ -4027,27 +4027,27 @@
         <v>-1</v>
       </c>
       <c r="V9" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W9" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X9" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y9" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D10" s="38">
         <v>-1</v>
@@ -4104,27 +4104,27 @@
         <v>-1</v>
       </c>
       <c r="V10" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W10" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X10" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y10" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B11" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D11" s="38">
         <v>-1</v>
@@ -4181,27 +4181,27 @@
         <v>-1</v>
       </c>
       <c r="V11" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W11" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X11" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y11" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D12" s="38">
         <v>-1</v>
@@ -4258,27 +4258,27 @@
         <v>-1</v>
       </c>
       <c r="V12" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W12" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X12" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y12" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B13" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D13" s="38">
         <v>-1</v>
@@ -4335,27 +4335,27 @@
         <v>-1</v>
       </c>
       <c r="V13" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W13" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X13" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y13" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B14" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D14" s="38">
         <v>-1</v>
@@ -4412,27 +4412,27 @@
         <v>-1</v>
       </c>
       <c r="V14" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W14" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X14" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y14" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B15" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C15" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D15" s="38">
         <v>-1</v>
@@ -4489,27 +4489,27 @@
         <v>-1</v>
       </c>
       <c r="V15" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W15" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X15" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y15" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B16" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D16" s="38">
         <v>-1</v>
@@ -4566,27 +4566,27 @@
         <v>-1</v>
       </c>
       <c r="V16" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W16" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X16" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y16" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B17" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D17" s="38">
         <v>-1</v>
@@ -4643,16 +4643,16 @@
         <v>-1</v>
       </c>
       <c r="V17" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="W17" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="X17" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Y17" s="38" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
@@ -4685,7 +4685,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="41" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
@@ -6858,13 +6858,13 @@
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" s="36" t="s">
+        <v>112</v>
+      </c>
+      <c r="N6" s="34" t="s">
         <v>113</v>
       </c>
-      <c r="N6" s="34" t="s">
+      <c r="O6" s="34" t="s">
         <v>114</v>
-      </c>
-      <c r="O6" s="34" t="s">
-        <v>115</v>
       </c>
       <c r="P6" s="1"/>
       <c r="Q6" s="1" t="e">
@@ -6979,7 +6979,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="Q8" s="1" t="e">
         <f>-(F8-I$8)</f>
@@ -7151,7 +7151,7 @@
         <v>0</v>
       </c>
       <c r="S12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -7785,7 +7785,7 @@
     <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H2" s="47" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I2" s="47"/>
       <c r="J2" s="47"/>
@@ -7795,12 +7795,12 @@
         <v>0</v>
       </c>
       <c r="M2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E3" s="22"/>
       <c r="F3" s="22" t="s">
@@ -7816,13 +7816,13 @@
         <v>33</v>
       </c>
       <c r="J3" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="K3" s="22" t="s">
         <v>117</v>
       </c>
-      <c r="K3" s="22" t="s">
+      <c r="L3" s="22" t="s">
         <v>118</v>
-      </c>
-      <c r="L3" s="22" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -8235,7 +8235,7 @@
         <v>5</v>
       </c>
       <c r="E11" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="3:6" x14ac:dyDescent="0.25">
@@ -8243,7 +8243,7 @@
         <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="3:6" x14ac:dyDescent="0.25">
@@ -8259,7 +8259,7 @@
         <v>9</v>
       </c>
       <c r="E14" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="15" spans="3:6" x14ac:dyDescent="0.25">
@@ -8275,7 +8275,7 @@
         <v>11</v>
       </c>
       <c r="E16" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>